<commit_message>
Add the 2026-27 schedule, next-game hero line, and league marks
- Schedule sheet (G, Date, H/A, Opp, Time (ET)) from the supplied calendar PDF;
  83 games as listed, flagged in CLAUDE.md
- Hero: next game with date and time, NHL shield and Eastern Conference marks
- Schedule tab grouped by month, next game highlighted
- CLAUDE.md: schedule schema, sortable-tables-with-locked-totals rule

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NVb2Bgn2cLfMh9qQ2WTHWv
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -14,8 +14,9 @@
     <sheet name="Cap" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Front Office" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="Trades" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Teams" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Notes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Schedule" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Teams" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Notes" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3605,6 +3606,88 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Seeded from franchise screens: owner goals, budget, cap, contracts, lines, two trade offers (both declined).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Goalie contracts (Sorokin, Varlamov) pending from the user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Varlamov sits in goalie slot 1 on the lineup screen, Sorokin in slot 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Schedule loaded from the sportsbrackets.net 2026-27 calendar PDF. It lists 83 games (42 home): 4 vs every Metropolitan club, 2 vs TOR. Reconcile against the game's calendar.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
@@ -5762,6 +5845,2136 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
+  <dimension ref="A1:E85"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="6" customWidth="1" min="3" max="3"/>
+    <col width="6" customWidth="1" min="4" max="4"/>
+    <col width="11" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>H/A</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Time (ET)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>3</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>10/08/2026</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>4</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>10/10/2026</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>10/13/2026</t>
+        </is>
+      </c>
+      <c r="C7" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D7" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>7:45p</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="n">
+        <v>6</v>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>10/15/2026</t>
+        </is>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" t="inlineStr">
+        <is>
+          <t>10/17/2026</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>10/20/2026</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>9</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>10/22/2026</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>10</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>10/25/2026</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>6p</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="n">
+        <v>11</v>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>10/27/2026</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>8p</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="n">
+        <v>12</v>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>10/29/2026</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>8p</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="n">
+        <v>13</v>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>10/31/2026</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>3:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="n">
+        <v>14</v>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>11/05/2026</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="n">
+        <v>15</v>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>11/07/2026</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="n">
+        <v>16</v>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>11/09/2026</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="n">
+        <v>17</v>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>11/12/2026</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>LAK</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="n">
+        <v>18</v>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>11/14/2026</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>ANA</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="n">
+        <v>19</v>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>11/17/2026</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="n">
+        <v>20</v>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>11/19/2026</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>8p</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="n">
+        <v>21</v>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>11/21/2026</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="n">
+        <v>22</v>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>11/23/2026</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="n">
+        <v>23</v>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>11/25/2026</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="n">
+        <v>24</v>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>11/27/2026</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>WPG</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="n">
+        <v>25</v>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>11/28/2026</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="n">
+        <v>26</v>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>12/01/2026</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="n">
+        <v>27</v>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>12/03/2026</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="n">
+        <v>28</v>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>12/04/2026</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>SJS</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="n">
+        <v>29</v>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>12/07/2026</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="n">
+        <v>30</v>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>12/10/2026</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="n">
+        <v>31</v>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>12/11/2026</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="n">
+        <v>32</v>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>12/15/2026</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>9p</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="n">
+        <v>33</v>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>12/16/2026</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>COL</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>9p</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="n">
+        <v>34</v>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>12/18/2026</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="n">
+        <v>35</v>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>12/20/2026</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="n">
+        <v>36</v>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>12/22/2026</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="n">
+        <v>37</v>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>12/26/2026</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>38</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>12/27/2026</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>39</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>12/30/2026</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>4p</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>40</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>01/02/2027</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>41</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>01/05/2027</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>VAN</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>10p</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>42</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>01/07/2027</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>CGY</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>9p</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>43</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>01/09/2027</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>EDM</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>4:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="n">
+        <v>44</v>
+      </c>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>01/13/2027</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D46" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="E46" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" t="n">
+        <v>45</v>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>01/15/2027</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>DAL</t>
+        </is>
+      </c>
+      <c r="E47" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="n">
+        <v>46</v>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>01/16/2027</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="E48" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="n">
+        <v>47</v>
+      </c>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>01/18/2027</t>
+        </is>
+      </c>
+      <c r="C49" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D49" t="inlineStr">
+        <is>
+          <t>NSH</t>
+        </is>
+      </c>
+      <c r="E49" t="inlineStr">
+        <is>
+          <t>3p</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="n">
+        <v>48</v>
+      </c>
+      <c r="B50" t="inlineStr">
+        <is>
+          <t>01/20/2027</t>
+        </is>
+      </c>
+      <c r="C50" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D50" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="E50" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51" t="n">
+        <v>49</v>
+      </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>01/22/2027</t>
+        </is>
+      </c>
+      <c r="C51" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D51" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E51" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="n">
+        <v>50</v>
+      </c>
+      <c r="B52" t="inlineStr">
+        <is>
+          <t>01/23/2027</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D52" t="inlineStr">
+        <is>
+          <t>SEA</t>
+        </is>
+      </c>
+      <c r="E52" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" t="n">
+        <v>51</v>
+      </c>
+      <c r="B53" t="inlineStr">
+        <is>
+          <t>01/26/2027</t>
+        </is>
+      </c>
+      <c r="C53" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D53" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="E53" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="n">
+        <v>52</v>
+      </c>
+      <c r="B54" t="inlineStr">
+        <is>
+          <t>01/28/2027</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D54" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="E54" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55" t="n">
+        <v>53</v>
+      </c>
+      <c r="B55" t="inlineStr">
+        <is>
+          <t>01/30/2027</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D55" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="E55" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56" t="n">
+        <v>54</v>
+      </c>
+      <c r="B56" t="inlineStr">
+        <is>
+          <t>02/01/2027</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D56" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="E56" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="n">
+        <v>55</v>
+      </c>
+      <c r="B57" t="inlineStr">
+        <is>
+          <t>02/03/2027</t>
+        </is>
+      </c>
+      <c r="C57" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D57" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="E57" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="n">
+        <v>56</v>
+      </c>
+      <c r="B58" t="inlineStr">
+        <is>
+          <t>02/12/2027</t>
+        </is>
+      </c>
+      <c r="C58" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D58" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="E58" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" t="n">
+        <v>57</v>
+      </c>
+      <c r="B59" t="inlineStr">
+        <is>
+          <t>02/13/2027</t>
+        </is>
+      </c>
+      <c r="C59" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D59" t="inlineStr">
+        <is>
+          <t>MIN</t>
+        </is>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" t="n">
+        <v>58</v>
+      </c>
+      <c r="B60" t="inlineStr">
+        <is>
+          <t>02/15/2027</t>
+        </is>
+      </c>
+      <c r="C60" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D60" t="inlineStr">
+        <is>
+          <t>UTA</t>
+        </is>
+      </c>
+      <c r="E60" t="inlineStr">
+        <is>
+          <t>3p</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" t="n">
+        <v>59</v>
+      </c>
+      <c r="B61" t="inlineStr">
+        <is>
+          <t>02/18/2027</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D61" t="inlineStr">
+        <is>
+          <t>NYR</t>
+        </is>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62" t="n">
+        <v>60</v>
+      </c>
+      <c r="B62" t="inlineStr">
+        <is>
+          <t>02/20/2027</t>
+        </is>
+      </c>
+      <c r="C62" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D62" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63" t="n">
+        <v>61</v>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>02/22/2027</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D63" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="n">
+        <v>62</v>
+      </c>
+      <c r="B64" t="inlineStr">
+        <is>
+          <t>02/23/2027</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D64" t="inlineStr">
+        <is>
+          <t>CHI</t>
+        </is>
+      </c>
+      <c r="E64" t="inlineStr">
+        <is>
+          <t>8p</t>
+        </is>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65" t="n">
+        <v>63</v>
+      </c>
+      <c r="B65" t="inlineStr">
+        <is>
+          <t>02/26/2027</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D65" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="E65" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" t="n">
+        <v>64</v>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>02/27/2027</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D66" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="n">
+        <v>65</v>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>03/01/2027</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D67" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="n">
+        <v>66</v>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>03/04/2027</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D68" t="inlineStr">
+        <is>
+          <t>VGK</t>
+        </is>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="n">
+        <v>67</v>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>03/07/2027</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D69" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>1p</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="n">
+        <v>68</v>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>03/09/2027</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D70" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="n">
+        <v>69</v>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>03/12/2027</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D71" t="inlineStr">
+        <is>
+          <t>FLA</t>
+        </is>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="n">
+        <v>70</v>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>03/13/2027</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D72" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="n">
+        <v>71</v>
+      </c>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>03/15/2027</t>
+        </is>
+      </c>
+      <c r="C73" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D73" t="inlineStr">
+        <is>
+          <t>BOS</t>
+        </is>
+      </c>
+      <c r="E73" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" t="n">
+        <v>72</v>
+      </c>
+      <c r="B74" t="inlineStr">
+        <is>
+          <t>03/17/2027</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D74" t="inlineStr">
+        <is>
+          <t>WSH</t>
+        </is>
+      </c>
+      <c r="E74" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" t="n">
+        <v>73</v>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>03/20/2027</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D75" t="inlineStr">
+        <is>
+          <t>PHI</t>
+        </is>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>3p</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="n">
+        <v>74</v>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>03/21/2027</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D76" t="inlineStr">
+        <is>
+          <t>BUF</t>
+        </is>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>3p</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="n">
+        <v>75</v>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>03/25/2027</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D77" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="E77" t="inlineStr">
+        <is>
+          <t>8p</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="n">
+        <v>76</v>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>03/27/2027</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D78" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="E78" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="n">
+        <v>77</v>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>03/30/2027</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D79" t="inlineStr">
+        <is>
+          <t>CAR</t>
+        </is>
+      </c>
+      <c r="E79" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="n">
+        <v>78</v>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>04/01/2027</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D80" t="inlineStr">
+        <is>
+          <t>PIT</t>
+        </is>
+      </c>
+      <c r="E80" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="n">
+        <v>79</v>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>04/02/2027</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D81" t="inlineStr">
+        <is>
+          <t>OTT</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="n">
+        <v>80</v>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>04/04/2027</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D82" t="inlineStr">
+        <is>
+          <t>MTL</t>
+        </is>
+      </c>
+      <c r="E82" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="n">
+        <v>81</v>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>04/06/2027</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D83" t="inlineStr">
+        <is>
+          <t>DET</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr">
+        <is>
+          <t>7:30p</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="n">
+        <v>82</v>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>04/08/2027</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D84" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="E84" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="A85" t="n">
+        <v>83</v>
+      </c>
+      <c r="B85" t="inlineStr">
+        <is>
+          <t>04/10/2027</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>H</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>CBJ</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>5p</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
   <dimension ref="A1:D34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -6506,74 +8719,4 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
-</file>
-
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Seeded from franchise screens: owner goals, budget, cap, contracts, lines, two trade offers (both declined).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Goalie contracts (Sorokin, Varlamov) pending from the user.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Varlamov sits in goalie slot 1 on the lineup screen, Sorokin in slot 2.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
 </file>
</xml_diff>

<commit_message>
Correct the schedule to the official 84-game 2026-27 season
The earlier load came from a third-party calendar PDF that omitted the
September opener, leaving 83 games. Replaced with the NHL.com release:
84 games, 42 home, opening 09/30/2026 at TOR. Every other game matched.
Pace math and the season count move from 82 to 84 per the new CBA.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01NVb2Bgn2cLfMh9qQ2WTHWv
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -3679,7 +3679,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Schedule loaded from the sportsbrackets.net 2026-27 calendar PDF. It lists 83 games (42 home): 4 vs every Metropolitan club, 2 vs TOR. Reconcile against the game's calendar.</t>
+          <t>Schedule loaded from the NHL.com official 2026-27 release: 84 games, 42 home, 42 away. The new CBA expands the season from 82 to 84; both added games are intra-division, so every Metropolitan rival is played 4 times. Opener is 09/30/2026 at TOR.</t>
         </is>
       </c>
     </row>
@@ -5845,7 +5845,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E85"/>
+  <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -5895,17 +5895,17 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>10/03/2026</t>
+          <t>09/30/2026</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -5920,22 +5920,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>10/06/2026</t>
+          <t>10/03/2026</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -5945,22 +5945,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>10/08/2026</t>
+          <t>10/06/2026</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -5970,7 +5970,7 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>10/10/2026</t>
+          <t>10/08/2026</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
@@ -5980,7 +5980,7 @@
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -5995,7 +5995,7 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>10/13/2026</t>
+          <t>10/10/2026</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
@@ -6005,12 +6005,12 @@
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>VAN</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>7:45p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -6020,22 +6020,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>10/15/2026</t>
+          <t>10/13/2026</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>VAN</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:45p</t>
         </is>
       </c>
     </row>
@@ -6045,7 +6045,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>10/17/2026</t>
+          <t>10/15/2026</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -6055,7 +6055,7 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -6070,17 +6070,17 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>10/20/2026</t>
+          <t>10/17/2026</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>ANA</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -6095,7 +6095,7 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>10/22/2026</t>
+          <t>10/20/2026</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
@@ -6105,12 +6105,12 @@
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>LAK</t>
+          <t>ANA</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6120,22 +6120,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>10/25/2026</t>
+          <t>10/22/2026</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>LAK</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>6p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -6145,7 +6145,7 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>10/27/2026</t>
+          <t>10/25/2026</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
@@ -6155,12 +6155,12 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>NSH</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>8p</t>
+          <t>6p</t>
         </is>
       </c>
     </row>
@@ -6170,7 +6170,7 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>10/29/2026</t>
+          <t>10/27/2026</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
@@ -6180,7 +6180,7 @@
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NSH</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
@@ -6195,22 +6195,22 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>10/31/2026</t>
+          <t>10/29/2026</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>3:30p</t>
+          <t>8p</t>
         </is>
       </c>
     </row>
@@ -6220,7 +6220,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>11/05/2026</t>
+          <t>10/31/2026</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -6230,12 +6230,12 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>3:30p</t>
         </is>
       </c>
     </row>
@@ -6245,7 +6245,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>11/07/2026</t>
+          <t>11/05/2026</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
@@ -6255,7 +6255,7 @@
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
@@ -6270,22 +6270,22 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>11/09/2026</t>
+          <t>11/07/2026</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6295,7 +6295,7 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>11/12/2026</t>
+          <t>11/09/2026</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
@@ -6305,7 +6305,7 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>LAK</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -6320,7 +6320,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>11/14/2026</t>
+          <t>11/12/2026</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -6330,7 +6330,7 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ANA</t>
+          <t>LAK</t>
         </is>
       </c>
       <c r="E20" t="inlineStr">
@@ -6345,22 +6345,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>11/17/2026</t>
+          <t>11/14/2026</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>CBJ</t>
+          <t>ANA</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>10p</t>
         </is>
       </c>
     </row>
@@ -6370,22 +6370,22 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>11/19/2026</t>
+          <t>11/17/2026</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>8p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6395,7 +6395,7 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>11/21/2026</t>
+          <t>11/19/2026</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
@@ -6405,12 +6405,12 @@
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>8p</t>
         </is>
       </c>
     </row>
@@ -6420,22 +6420,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>11/23/2026</t>
+          <t>11/21/2026</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>TOR</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6445,7 +6445,7 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>11/25/2026</t>
+          <t>11/23/2026</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
@@ -6455,12 +6455,12 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>TOR</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -6470,7 +6470,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>11/27/2026</t>
+          <t>11/25/2026</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -6480,12 +6480,12 @@
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>WPG</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6495,17 +6495,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>11/28/2026</t>
+          <t>11/27/2026</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>WPG</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -6520,22 +6520,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>12/01/2026</t>
+          <t>11/28/2026</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -6545,17 +6545,17 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>12/03/2026</t>
+          <t>12/01/2026</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
@@ -6570,17 +6570,17 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>12/04/2026</t>
+          <t>12/03/2026</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>SJS</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
@@ -6595,7 +6595,7 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>12/07/2026</t>
+          <t>12/04/2026</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
@@ -6605,12 +6605,12 @@
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>SJS</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6620,7 +6620,7 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>12/10/2026</t>
+          <t>12/07/2026</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -6630,12 +6630,12 @@
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>1p</t>
         </is>
       </c>
     </row>
@@ -6645,17 +6645,17 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>12/11/2026</t>
+          <t>12/10/2026</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="E33" t="inlineStr">
@@ -6670,7 +6670,7 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>12/15/2026</t>
+          <t>12/11/2026</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -6680,12 +6680,12 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>UTA</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>9p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6695,7 +6695,7 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>12/16/2026</t>
+          <t>12/15/2026</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -6705,7 +6705,7 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>COL</t>
+          <t>UTA</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -6720,7 +6720,7 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>12/18/2026</t>
+          <t>12/16/2026</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -6730,12 +6730,12 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>VGK</t>
+          <t>COL</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>9p</t>
         </is>
       </c>
     </row>
@@ -6745,22 +6745,22 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>12/20/2026</t>
+          <t>12/18/2026</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>VGK</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>10p</t>
         </is>
       </c>
     </row>
@@ -6770,7 +6770,7 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>12/22/2026</t>
+          <t>12/20/2026</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -6780,7 +6780,7 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
@@ -6795,12 +6795,12 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>12/26/2026</t>
+          <t>12/22/2026</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
@@ -6820,17 +6820,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>12/27/2026</t>
+          <t>12/26/2026</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -6845,7 +6845,7 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>12/30/2026</t>
+          <t>12/27/2026</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -6855,12 +6855,12 @@
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
         <is>
-          <t>4p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -6870,22 +6870,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>01/02/2027</t>
+          <t>12/30/2026</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>10p</t>
+          <t>4p</t>
         </is>
       </c>
     </row>
@@ -6895,7 +6895,7 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>01/05/2027</t>
+          <t>01/02/2027</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -6905,7 +6905,7 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>VAN</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E43" t="inlineStr">
@@ -6920,7 +6920,7 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>01/07/2027</t>
+          <t>01/05/2027</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -6930,7 +6930,7 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>CGY</t>
+          <t>VAN</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
@@ -6945,7 +6945,7 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>01/09/2027</t>
+          <t>01/07/2027</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -6955,12 +6955,12 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>EDM</t>
+          <t>CGY</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
         <is>
-          <t>4:30p</t>
+          <t>8p</t>
         </is>
       </c>
     </row>
@@ -6970,22 +6970,22 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>01/13/2027</t>
+          <t>01/09/2027</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>EDM</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>3:30p</t>
         </is>
       </c>
     </row>
@@ -6995,7 +6995,7 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>01/15/2027</t>
+          <t>01/13/2027</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
@@ -7005,12 +7005,12 @@
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>DAL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -7020,17 +7020,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>01/16/2027</t>
+          <t>01/15/2027</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>DAL</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -7045,22 +7045,22 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>01/18/2027</t>
+          <t>01/16/2027</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>NSH</t>
+          <t>NJD</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>3p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7070,7 +7070,7 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>01/20/2027</t>
+          <t>01/18/2027</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
@@ -7080,12 +7080,12 @@
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>NSH</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>3p</t>
         </is>
       </c>
     </row>
@@ -7095,17 +7095,17 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>01/22/2027</t>
+          <t>01/20/2027</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
@@ -7120,22 +7120,22 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>01/23/2027</t>
+          <t>01/22/2027</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>SEA</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7145,22 +7145,22 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>01/26/2027</t>
+          <t>01/23/2027</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>SEA</t>
         </is>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -7170,7 +7170,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>01/28/2027</t>
+          <t>01/26/2027</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -7180,7 +7180,7 @@
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -7195,7 +7195,7 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>01/30/2027</t>
+          <t>01/28/2027</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -7205,7 +7205,7 @@
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -7220,7 +7220,7 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>02/01/2027</t>
+          <t>01/30/2027</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -7230,12 +7230,12 @@
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7245,7 +7245,7 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>02/03/2027</t>
+          <t>02/01/2027</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -7255,12 +7255,12 @@
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>1p</t>
         </is>
       </c>
     </row>
@@ -7270,7 +7270,7 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>02/12/2027</t>
+          <t>02/03/2027</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -7280,7 +7280,7 @@
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -7295,17 +7295,17 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>02/13/2027</t>
+          <t>02/12/2027</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>MIN</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="E59" t="inlineStr">
@@ -7320,7 +7320,7 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>02/15/2027</t>
+          <t>02/13/2027</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -7330,12 +7330,12 @@
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>UTA</t>
+          <t>MIN</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>3p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7345,7 +7345,7 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>02/18/2027</t>
+          <t>02/15/2027</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -7355,12 +7355,12 @@
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>NYR</t>
+          <t>UTA</t>
         </is>
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>3p</t>
         </is>
       </c>
     </row>
@@ -7370,17 +7370,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>02/20/2027</t>
+          <t>02/18/2027</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>NYR</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -7395,7 +7395,7 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>02/22/2027</t>
+          <t>02/20/2027</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
@@ -7405,7 +7405,7 @@
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>CBJ</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -7420,7 +7420,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>02/23/2027</t>
+          <t>02/22/2027</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -7430,12 +7430,12 @@
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>CHI</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>8p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7445,22 +7445,22 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>02/26/2027</t>
+          <t>02/23/2027</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>CHI</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>8p</t>
         </is>
       </c>
     </row>
@@ -7470,17 +7470,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>02/27/2027</t>
+          <t>02/26/2027</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>CBJ</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -7495,17 +7495,17 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>03/01/2027</t>
+          <t>02/27/2027</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>CBJ</t>
         </is>
       </c>
       <c r="E67" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>03/04/2027</t>
+          <t>03/01/2027</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -7530,7 +7530,7 @@
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>VGK</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -7545,7 +7545,7 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>03/07/2027</t>
+          <t>03/04/2027</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -7555,12 +7555,12 @@
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>VGK</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>1p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7570,7 +7570,7 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>03/09/2027</t>
+          <t>03/07/2027</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -7580,12 +7580,12 @@
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>1p</t>
         </is>
       </c>
     </row>
@@ -7595,17 +7595,17 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>03/12/2027</t>
+          <t>03/09/2027</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>FLA</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
@@ -7620,7 +7620,7 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>03/13/2027</t>
+          <t>03/12/2027</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -7630,7 +7630,7 @@
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>TBL</t>
+          <t>FLA</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
@@ -7645,7 +7645,7 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>03/15/2027</t>
+          <t>03/13/2027</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
@@ -7655,7 +7655,7 @@
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>BOS</t>
+          <t>TBL</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -7670,7 +7670,7 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>03/17/2027</t>
+          <t>03/15/2027</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -7680,7 +7680,7 @@
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>WSH</t>
+          <t>BOS</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
@@ -7695,22 +7695,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>03/20/2027</t>
+          <t>03/17/2027</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>PHI</t>
+          <t>WSH</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>3p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7720,7 +7720,7 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>03/21/2027</t>
+          <t>03/20/2027</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
@@ -7730,7 +7730,7 @@
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>BUF</t>
+          <t>PHI</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
@@ -7745,22 +7745,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>03/25/2027</t>
+          <t>03/21/2027</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>STL</t>
+          <t>BUF</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>8p</t>
+          <t>3p</t>
         </is>
       </c>
     </row>
@@ -7770,22 +7770,22 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>03/27/2027</t>
+          <t>03/25/2027</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>STL</t>
         </is>
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>8p</t>
         </is>
       </c>
     </row>
@@ -7795,7 +7795,7 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>03/30/2027</t>
+          <t>03/27/2027</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
@@ -7805,12 +7805,12 @@
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>CAR</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -7820,17 +7820,17 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>04/01/2027</t>
+          <t>03/30/2027</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>PIT</t>
+          <t>CAR</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
@@ -7845,17 +7845,17 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>04/02/2027</t>
+          <t>04/01/2027</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>H</t>
+          <t>A</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>OTT</t>
+          <t>PIT</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
@@ -7870,7 +7870,7 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>04/04/2027</t>
+          <t>04/02/2027</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
@@ -7880,12 +7880,12 @@
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>MTL</t>
+          <t>OTT</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>7:30p</t>
+          <t>7p</t>
         </is>
       </c>
     </row>
@@ -7895,7 +7895,7 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>04/06/2027</t>
+          <t>04/04/2027</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
@@ -7905,7 +7905,7 @@
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>DET</t>
+          <t>MTL</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
@@ -7920,22 +7920,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>04/08/2027</t>
+          <t>04/06/2027</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>A</t>
+          <t>H</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>NJD</t>
+          <t>DET</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>7p</t>
+          <t>7:30p</t>
         </is>
       </c>
     </row>
@@ -7945,20 +7945,45 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
+          <t>04/08/2027</t>
+        </is>
+      </c>
+      <c r="C85" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="D85" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="E85" t="inlineStr">
+        <is>
+          <t>7p</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="A86" t="n">
+        <v>84</v>
+      </c>
+      <c r="B86" t="inlineStr">
+        <is>
           <t>04/10/2027</t>
         </is>
       </c>
-      <c r="C85" t="inlineStr">
+      <c r="C86" t="inlineStr">
         <is>
           <t>H</t>
         </is>
       </c>
-      <c r="D85" t="inlineStr">
+      <c r="D86" t="inlineStr">
         <is>
           <t>CBJ</t>
         </is>
       </c>
-      <c r="E85" t="inlineStr">
+      <c r="E86" t="inlineStr">
         <is>
           <t>5p</t>
         </is>

</xml_diff>

<commit_message>
Log G1 at TOR and add player cards (20260907-025218)
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -17,6 +17,14 @@
     <sheet name="Schedule" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="Teams" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="Notes" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Games" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Scoring" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Goalie Game Log" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Opp Goaltending" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Skater Game Log" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Recaps" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Inside" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Headlines" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3612,7 +3620,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B6"/>
+  <dimension ref="A1:B7"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -3680,6 +3688,1421 @@
       <c r="B6" t="inlineStr">
         <is>
           <t>Schedule loaded from the NHL.com official 2026-27 release: 84 games, 42 home, 42 away. The new CBA expands the season from 82 to 84; both added games are intra-division, so every Metropolitan rival is played 4 times. Opener is 09/30/2026 at TOR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>G1 at TOR: Skater box score pending; Horvat's goal and the three NYI minors are the only per-player figures the play-by-play supports.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:AL3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="7" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="9" customWidth="1" min="18" max="18"/>
+    <col width="9" customWidth="1" min="19" max="19"/>
+    <col width="8" customWidth="1" min="20" max="20"/>
+    <col width="8" customWidth="1" min="21" max="21"/>
+    <col width="7" customWidth="1" min="22" max="22"/>
+    <col width="7" customWidth="1" min="23" max="23"/>
+    <col width="9" customWidth="1" min="24" max="24"/>
+    <col width="9" customWidth="1" min="25" max="25"/>
+    <col width="7" customWidth="1" min="26" max="26"/>
+    <col width="7" customWidth="1" min="27" max="27"/>
+    <col width="7" customWidth="1" min="28" max="28"/>
+    <col width="7" customWidth="1" min="29" max="29"/>
+    <col width="7" customWidth="1" min="30" max="30"/>
+    <col width="7" customWidth="1" min="31" max="31"/>
+    <col width="7" customWidth="1" min="32" max="32"/>
+    <col width="7" customWidth="1" min="33" max="33"/>
+    <col width="7" customWidth="1" min="34" max="34"/>
+    <col width="7" customWidth="1" min="35" max="35"/>
+    <col width="8" customWidth="1" min="36" max="36"/>
+    <col width="8" customWidth="1" min="37" max="37"/>
+    <col width="9" customWidth="1" min="38" max="38"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>H/A</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>GF</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>P1 F</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>P1 A</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>P2 F</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>P2 A</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>P3 F</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>P3 A</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>OT F</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>OT A</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>SO F</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>SO A</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>Shots F</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>Shots A</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>Hits F</t>
+        </is>
+      </c>
+      <c r="U1" s="1" t="inlineStr">
+        <is>
+          <t>Hits A</t>
+        </is>
+      </c>
+      <c r="V1" s="1" t="inlineStr">
+        <is>
+          <t>TOA F</t>
+        </is>
+      </c>
+      <c r="W1" s="1" t="inlineStr">
+        <is>
+          <t>TOA A</t>
+        </is>
+      </c>
+      <c r="X1" s="1" t="inlineStr">
+        <is>
+          <t>Pass% F</t>
+        </is>
+      </c>
+      <c r="Y1" s="1" t="inlineStr">
+        <is>
+          <t>Pass% A</t>
+        </is>
+      </c>
+      <c r="Z1" s="1" t="inlineStr">
+        <is>
+          <t>FOW F</t>
+        </is>
+      </c>
+      <c r="AA1" s="1" t="inlineStr">
+        <is>
+          <t>FOW A</t>
+        </is>
+      </c>
+      <c r="AB1" s="1" t="inlineStr">
+        <is>
+          <t>PIM F</t>
+        </is>
+      </c>
+      <c r="AC1" s="1" t="inlineStr">
+        <is>
+          <t>PIM A</t>
+        </is>
+      </c>
+      <c r="AD1" s="1" t="inlineStr">
+        <is>
+          <t>PP F</t>
+        </is>
+      </c>
+      <c r="AE1" s="1" t="inlineStr">
+        <is>
+          <t>PP A</t>
+        </is>
+      </c>
+      <c r="AF1" s="1" t="inlineStr">
+        <is>
+          <t>PPM F</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>PPM A</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
+          <t>SHG F</t>
+        </is>
+      </c>
+      <c r="AI1" s="1" t="inlineStr">
+        <is>
+          <t>SHG A</t>
+        </is>
+      </c>
+      <c r="AJ1" s="1" t="inlineStr">
+        <is>
+          <t>Streak</t>
+        </is>
+      </c>
+      <c r="AK1" s="1" t="inlineStr">
+        <is>
+          <t>Record</t>
+        </is>
+      </c>
+      <c r="AL1" s="1" t="inlineStr">
+        <is>
+          <t>Summary</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+      <c r="U2" s="2" t="n"/>
+      <c r="V2" s="2" t="n"/>
+      <c r="W2" s="2" t="n"/>
+      <c r="X2" s="2" t="n"/>
+      <c r="Y2" s="2" t="n"/>
+      <c r="Z2" s="2" t="n"/>
+      <c r="AA2" s="2" t="n"/>
+      <c r="AB2" s="2" t="n"/>
+      <c r="AC2" s="2" t="n"/>
+      <c r="AD2" s="2" t="n"/>
+      <c r="AE2" s="2" t="n"/>
+      <c r="AF2" s="2" t="n"/>
+      <c r="AG2" s="2" t="n"/>
+      <c r="AH2" s="2" t="n"/>
+      <c r="AI2" s="2" t="n"/>
+      <c r="AJ2" s="2" t="n"/>
+      <c r="AK2" s="2" t="n"/>
+      <c r="AL2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>OTL</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>1</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>1</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>1</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0</v>
+      </c>
+      <c r="R3" t="n">
+        <v>32</v>
+      </c>
+      <c r="S3" t="n">
+        <v>43</v>
+      </c>
+      <c r="T3" t="n">
+        <v>28</v>
+      </c>
+      <c r="U3" t="n">
+        <v>37</v>
+      </c>
+      <c r="V3" t="inlineStr">
+        <is>
+          <t>07:06</t>
+        </is>
+      </c>
+      <c r="W3" t="inlineStr">
+        <is>
+          <t>05:15</t>
+        </is>
+      </c>
+      <c r="X3" t="n">
+        <v>71.59999999999999</v>
+      </c>
+      <c r="Y3" t="n">
+        <v>88.09999999999999</v>
+      </c>
+      <c r="Z3" t="n">
+        <v>21</v>
+      </c>
+      <c r="AA3" t="n">
+        <v>16</v>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>04:00</t>
+        </is>
+      </c>
+      <c r="AD3" t="inlineStr">
+        <is>
+          <t>0/2</t>
+        </is>
+      </c>
+      <c r="AE3" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="AF3" t="inlineStr">
+        <is>
+          <t>02:48</t>
+        </is>
+      </c>
+      <c r="AG3" t="inlineStr">
+        <is>
+          <t>04:48</t>
+        </is>
+      </c>
+      <c r="AH3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AI3" t="n">
+        <v>0</v>
+      </c>
+      <c r="AJ3" t="inlineStr">
+        <is>
+          <t>OT1</t>
+        </is>
+      </c>
+      <c r="AK3" t="inlineStr">
+        <is>
+          <t>0-0-1</t>
+        </is>
+      </c>
+      <c r="AL3" t="inlineStr">
+        <is>
+          <t>Gut punch OTL on the road to start the year. Isles look strong all game but wither when it counts.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:I5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Team</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Scorer</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>A1</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>A2</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>Score</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>NYI</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>B. Horvat</t>
+        </is>
+      </c>
+      <c r="H3" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>1-0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>B. Duhaime</t>
+        </is>
+      </c>
+      <c r="H4" t="inlineStr">
+        <is>
+          <t>EV</t>
+        </is>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>1-1</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>J. Roslovic</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
+        <is>
+          <t>GWG</t>
+        </is>
+      </c>
+      <c r="I5" t="inlineStr">
+        <is>
+          <t>1-2</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Goalie</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>SV%</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>TOI</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>SO</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Start/Relief</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>I. Sorokin</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>OTL</t>
+        </is>
+      </c>
+      <c r="E3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G3" t="n">
+        <v>2</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0.953</v>
+      </c>
+      <c r="I3" t="inlineStr">
+        <is>
+          <t>65:00</t>
+        </is>
+      </c>
+      <c r="J3" t="n">
+        <v>0</v>
+      </c>
+      <c r="K3" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:J3"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="9" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Goalie</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Catches</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Dec</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>SA</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>SV</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>GA</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>SV%</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>TOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>M. Stolarz</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="F3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G3" t="n">
+        <v>31</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.969</v>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>65:00</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:T2"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+    <col width="7" customWidth="1" min="5" max="5"/>
+    <col width="7" customWidth="1" min="6" max="6"/>
+    <col width="7" customWidth="1" min="7" max="7"/>
+    <col width="7" customWidth="1" min="8" max="8"/>
+    <col width="7" customWidth="1" min="9" max="9"/>
+    <col width="7" customWidth="1" min="10" max="10"/>
+    <col width="7" customWidth="1" min="11" max="11"/>
+    <col width="7" customWidth="1" min="12" max="12"/>
+    <col width="7" customWidth="1" min="13" max="13"/>
+    <col width="7" customWidth="1" min="14" max="14"/>
+    <col width="7" customWidth="1" min="15" max="15"/>
+    <col width="7" customWidth="1" min="16" max="16"/>
+    <col width="7" customWidth="1" min="17" max="17"/>
+    <col width="7" customWidth="1" min="18" max="18"/>
+    <col width="7" customWidth="1" min="19" max="19"/>
+    <col width="7" customWidth="1" min="20" max="20"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Player</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Pos</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>A</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Pts</t>
+        </is>
+      </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>+/-</t>
+        </is>
+      </c>
+      <c r="I1" s="1" t="inlineStr">
+        <is>
+          <t>SOG</t>
+        </is>
+      </c>
+      <c r="J1" s="1" t="inlineStr">
+        <is>
+          <t>PIM</t>
+        </is>
+      </c>
+      <c r="K1" s="1" t="inlineStr">
+        <is>
+          <t>Hits</t>
+        </is>
+      </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Blk</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>PPG</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>PPA</t>
+        </is>
+      </c>
+      <c r="O1" s="1" t="inlineStr">
+        <is>
+          <t>SHG</t>
+        </is>
+      </c>
+      <c r="P1" s="1" t="inlineStr">
+        <is>
+          <t>GWG</t>
+        </is>
+      </c>
+      <c r="Q1" s="1" t="inlineStr">
+        <is>
+          <t>ENG</t>
+        </is>
+      </c>
+      <c r="R1" s="1" t="inlineStr">
+        <is>
+          <t>FOW</t>
+        </is>
+      </c>
+      <c r="S1" s="1" t="inlineStr">
+        <is>
+          <t>FOL</t>
+        </is>
+      </c>
+      <c r="T1" s="1" t="inlineStr">
+        <is>
+          <t>TOI</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+      <c r="H2" s="2" t="n"/>
+      <c r="I2" s="2" t="n"/>
+      <c r="J2" s="2" t="n"/>
+      <c r="K2" s="2" t="n"/>
+      <c r="L2" s="2" t="n"/>
+      <c r="M2" s="2" t="n"/>
+      <c r="N2" s="2" t="n"/>
+      <c r="O2" s="2" t="n"/>
+      <c r="P2" s="2" t="n"/>
+      <c r="Q2" s="2" t="n"/>
+      <c r="R2" s="2" t="n"/>
+      <c r="S2" s="2" t="n"/>
+      <c r="T2" s="2" t="n"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:D6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="7" customWidth="1" min="1" max="1"/>
+    <col width="7" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="7" customWidth="1" min="4" max="4"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Opp</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Period</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Horvat picks up a loose puck over the blue line and dekes Stolarz at the right post (1-0). Ekman-Larsson slashing. Nylander is hauled down on a breakaway by Holmstrom and gets a penalty shot. Sorokin turns him away at the right post. Romanov slashing with two minutes left. Pelech slashes Paul with 7 seconds left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Nylander for slashing, 4-on-4 for 1:14. Barzal for slashing.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>3</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Duhaime gets a late break in the slot and has hands in close (1-1) with 3 minutes left.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>TOR</t>
+        </is>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>OT</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>Roslovic rebounds himself at the right post for the winner (2-1).</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="100" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Bullet</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>NYI led &lt;b&gt;1-0&lt;/b&gt; after the 1st in G1 at TOR and did not score again.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Toronto put &lt;b&gt;32 of its 43 shots (74%)&lt;/b&gt; on Sorokin after the first intermission.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>The Isles killed all &lt;b&gt;3&lt;/b&gt; Toronto power plays and went &lt;b&gt;0 for 2&lt;/b&gt; on their own.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Toronto out-hit NYI &lt;b&gt;37-28&lt;/b&gt; and completed &lt;b&gt;88.1%&lt;/b&gt; of its passes to the Isles' &lt;b&gt;71.6%&lt;/b&gt;.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E6"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="8" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="22" customWidth="1" min="3" max="3"/>
+    <col width="110" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>G</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Fig</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Kicker</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Text</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Tone</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="n">
+        <v>1</v>
+      </c>
+      <c r="B3" t="n">
+        <v>41</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>Saves</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Sorokin&lt;/b&gt; faced &lt;b&gt;43&lt;/b&gt; shots in G1 at TOR and was beaten only in the last 3 minutes of regulation and in overtime.</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>1</v>
+      </c>
+      <c r="B4" t="n">
+        <v>1</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Goals</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Horvat&lt;/b&gt; picked up a loose puck over the blue line and deked Stolarz at the right post to open the scoring.</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>Penalty shot stopped</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Nylander&lt;/b&gt; was hauled down by &lt;b&gt;Holmstrom&lt;/b&gt; on a breakaway in the 1st, and Sorokin turned him away at the right post.</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>active</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="n">
+        <v>1</v>
+      </c>
+      <c r="B6" t="n">
+        <v>3</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>Slashing minors</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>&lt;b&gt;Romanov&lt;/b&gt;, &lt;b&gt;Pelech&lt;/b&gt; and &lt;b&gt;Barzal&lt;/b&gt; each took one in G1 at TOR, and Toronto came away with nothing on the power play.</t>
+        </is>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>active</t>
         </is>
       </c>
     </row>
@@ -4921,7 +6344,6 @@
           <t>SCR</t>
         </is>
       </c>
-      <c r="B45" t="inlineStr"/>
       <c r="C45" t="inlineStr">
         <is>
           <t>C. Ritchie</t>
@@ -4942,7 +6364,6 @@
           <t>SCR</t>
         </is>
       </c>
-      <c r="B46" t="inlineStr"/>
       <c r="C46" t="inlineStr">
         <is>
           <t>T. DeAngelo</t>
@@ -4963,7 +6384,6 @@
           <t>SCR</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr"/>
       <c r="C47" t="inlineStr">
         <is>
           <t>K. MacLean</t>

</xml_diff>

<commit_message>
Widen Trades into Transactions and log the Deslauriers decline (20260907-025754)
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -13,18 +13,18 @@
     <sheet name="Budget" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Cap" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="Front Office" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Trades" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Schedule" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Teams" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Notes" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Games" sheetId="11" state="visible" r:id="rId11"/>
-    <sheet name="Scoring" sheetId="12" state="visible" r:id="rId12"/>
-    <sheet name="Goalie Game Log" sheetId="13" state="visible" r:id="rId13"/>
-    <sheet name="Opp Goaltending" sheetId="14" state="visible" r:id="rId14"/>
-    <sheet name="Skater Game Log" sheetId="15" state="visible" r:id="rId15"/>
-    <sheet name="Recaps" sheetId="16" state="visible" r:id="rId16"/>
-    <sheet name="Inside" sheetId="17" state="visible" r:id="rId17"/>
-    <sheet name="Headlines" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="Schedule" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Teams" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Notes" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Games" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Scoring" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Goalie Game Log" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="Opp Goaltending" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="Skater Game Log" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="Recaps" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="Inside" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="Headlines" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="Transactions" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -3620,100 +3620,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="44" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Note</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Seeded from franchise screens: owner goals, budget, cap, contracts, lines, two trade offers (both declined).</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Goalie contracts (Sorokin, Varlamov) pending from the user.</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B5" t="inlineStr">
-        <is>
-          <t>Varlamov sits in goalie slot 1 on the lineup screen, Sorokin in slot 2.</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B6" t="inlineStr">
-        <is>
-          <t>Schedule loaded from the NHL.com official 2026-27 release: 84 games, 42 home, 42 away. The new CBA expands the season from 82 to 84; both added games are intra-division, so every Metropolitan rival is played 4 times. Opener is 09/30/2026 at TOR.</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="inlineStr">
-        <is>
-          <t>09/30/2026</t>
-        </is>
-      </c>
-      <c r="B7" t="inlineStr">
-        <is>
-          <t>G1 at TOR: Skater box score pending; Horvat's goal and the three NYI minors are the only per-player figures the play-by-play supports.</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:AL3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -4140,7 +4046,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4328,7 +4234,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4470,7 +4376,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4602,7 +4508,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4762,7 +4668,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4890,7 +4796,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -4964,7 +4870,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -5103,6 +5009,186 @@
       <c r="E6" t="inlineStr">
         <is>
           <t>active</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G5"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="14" customWidth="1" min="2" max="2"/>
+    <col width="10" customWidth="1" min="3" max="3"/>
+    <col width="11" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="32" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
+          <t>Partner</t>
+        </is>
+      </c>
+      <c r="D1" s="1" t="inlineStr">
+        <is>
+          <t>Direction</t>
+        </is>
+      </c>
+      <c r="E1" s="1" t="inlineStr">
+        <is>
+          <t>Out</t>
+        </is>
+      </c>
+      <c r="F1" s="1" t="inlineStr">
+        <is>
+          <t>In</t>
+        </is>
+      </c>
+      <c r="G1" s="1" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="n"/>
+      <c r="D2" s="2" t="n"/>
+      <c r="E2" s="2" t="n"/>
+      <c r="F2" s="2" t="n"/>
+      <c r="G2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Trade offer</t>
+        </is>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>TBL</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>Incoming</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>NYI 2027 R3; I. George (D, $0.915M)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>TOR 2027 R4; TBL 2027 R4</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Trade offer</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>STL</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>Incoming</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>COL 2028 R3; J. Nurmi (LW, $0.870M)</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>STL 2028 R4; STL 2028 R7</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>Declined</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>Incoming</t>
+        </is>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>N. Deslauriers</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>Declined</t>
         </is>
       </c>
     </row>
@@ -7139,132 +7225,6 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F4"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="9" customWidth="1" min="2" max="2"/>
-    <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="36" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="10" customWidth="1" min="6" max="6"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Date</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Partner</t>
-        </is>
-      </c>
-      <c r="C1" s="1" t="inlineStr">
-        <is>
-          <t>Direction</t>
-        </is>
-      </c>
-      <c r="D1" s="1" t="inlineStr">
-        <is>
-          <t>Out</t>
-        </is>
-      </c>
-      <c r="E1" s="1" t="inlineStr">
-        <is>
-          <t>In</t>
-        </is>
-      </c>
-      <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Result</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="n"/>
-      <c r="B2" s="2" t="n"/>
-      <c r="C2" s="2" t="n"/>
-      <c r="D2" s="2" t="n"/>
-      <c r="E2" s="2" t="n"/>
-      <c r="F2" s="2" t="n"/>
-    </row>
-    <row r="3">
-      <c r="A3" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>TBL</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
-        <is>
-          <t>Incoming</t>
-        </is>
-      </c>
-      <c r="D3" t="inlineStr">
-        <is>
-          <t>NYI 2027 R3; I. George (D, $0.915M)</t>
-        </is>
-      </c>
-      <c r="E3" t="inlineStr">
-        <is>
-          <t>TOR 2027 R4; TBL 2027 R4</t>
-        </is>
-      </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>Declined</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" t="inlineStr">
-        <is>
-          <t>09/29/2026</t>
-        </is>
-      </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>STL</t>
-        </is>
-      </c>
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Incoming</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
-        <is>
-          <t>COL 2028 R3; J. Nurmi (LW, $0.870M)</t>
-        </is>
-      </c>
-      <c r="E4" t="inlineStr">
-        <is>
-          <t>STL 2028 R4; STL 2028 R7</t>
-        </is>
-      </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>Declined</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
   <dimension ref="A1:E86"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
@@ -9414,7 +9374,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -10164,4 +10124,110 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:B8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="44" customWidth="1" min="2" max="2"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="B1" s="1" t="inlineStr">
+        <is>
+          <t>Note</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="2" t="n"/>
+      <c r="B2" s="2" t="n"/>
+    </row>
+    <row r="3">
+      <c r="A3" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B3" t="inlineStr">
+        <is>
+          <t>Seeded from franchise screens: owner goals, budget, cap, contracts, lines, two trade offers (both declined).</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Goalie contracts (Sorokin, Varlamov) pending from the user.</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>Varlamov sits in goalie slot 1 on the lineup screen, Sorokin in slot 2.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" t="inlineStr">
+        <is>
+          <t>09/29/2026</t>
+        </is>
+      </c>
+      <c r="B6" t="inlineStr">
+        <is>
+          <t>Schedule loaded from the NHL.com official 2026-27 release: 84 games, 42 home, 42 away. The new CBA expands the season from 82 to 84; both added games are intra-division, so every Metropolitan rival is played 4 times. Opener is 09/30/2026 at TOR.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="B7" t="inlineStr">
+        <is>
+          <t>G1 at TOR: Skater box score pending; Horvat's goal and the three NYI minors are the only per-player figures the play-by-play supports.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" t="inlineStr">
+        <is>
+          <t>09/30/2026</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
+          <t>Declined N. Deslauriers. The source screen was not captured, so the type (trade offer, signing or waivers) and the counterparty are unrecorded.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Record the Deslauriers pass as a waivers row (20260907-030149)
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -5163,17 +5163,17 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
+          <t>Waivers</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
           <t>-</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Incoming</t>
+          <t>Claim</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -10223,7 +10223,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Declined N. Deslauriers. The source screen was not captured, so the type (trade offer, signing or waivers) and the counterparty are unrecorded.</t>
+          <t>Passed on N. Deslauriers on waivers. A waiver claim has no trade partner, so Partner stays '-'.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Rewrite the Horvat headline; open the scoring implied a sequence that never came (20260907-130814)
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -4831,7 +4831,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>NYI led &lt;b&gt;1-0&lt;/b&gt; after the 1st in G1 at TOR and did not score again.</t>
+          <t>NYI carried a &lt;b&gt;1-0&lt;/b&gt; lead into the 3rd in G1 at TOR and lost it with 3 minutes to play.</t>
         </is>
       </c>
     </row>
@@ -4957,7 +4957,7 @@
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Horvat&lt;/b&gt; picked up a loose puck over the blue line and deked Stolarz at the right post to open the scoring.</t>
+          <t>&lt;b&gt;Horvat&lt;/b&gt; picked up a loose puck over the blue line and deked Stolarz at the right post in the 1st of G1 at TOR, the only puck NYI got past him.</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">

</xml_diff>

<commit_message>
Top up G2 with the team-stats screens (20260908-030802)
The 1st, 2nd and final screens fill the Games row: 35-42 shots, 40-34 hits,
7:31-5:44 on attack, 14 of 46 faceoffs, 6:00-10:00 in penalties, PP 1/5, PK 3/3,
one shorthanded goal. Per-period shots and hits come from differencing the
cumulative screens. Rittich's 35 SA / 29 SV / 6 GA goes into Opp Goaltending.

PP 1/5 with the only power-play goal in the 3rd settles the open question from
the last pass: Cizikas' goal was even strength, so its EV label stands.

Two Inside bullets added now that the team stats exist - outshot 42-35 and 14 of
46 on the draw, and a season power play of 1 for 7 against a perfect kill.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gvmhg1m6TGt3JAtgHQ7SJs
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -4101,6 +4101,76 @@
       <c r="Q4" t="n">
         <v>0</v>
       </c>
+      <c r="R4" t="n">
+        <v>35</v>
+      </c>
+      <c r="S4" t="n">
+        <v>42</v>
+      </c>
+      <c r="T4" t="n">
+        <v>40</v>
+      </c>
+      <c r="U4" t="n">
+        <v>34</v>
+      </c>
+      <c r="V4" t="inlineStr">
+        <is>
+          <t>07:31</t>
+        </is>
+      </c>
+      <c r="W4" t="inlineStr">
+        <is>
+          <t>05:44</t>
+        </is>
+      </c>
+      <c r="X4" t="n">
+        <v>74.40000000000001</v>
+      </c>
+      <c r="Y4" t="n">
+        <v>89.2</v>
+      </c>
+      <c r="Z4" t="n">
+        <v>14</v>
+      </c>
+      <c r="AA4" t="n">
+        <v>32</v>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>06:00</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="AD4" t="inlineStr">
+        <is>
+          <t>1/5</t>
+        </is>
+      </c>
+      <c r="AE4" t="inlineStr">
+        <is>
+          <t>0/3</t>
+        </is>
+      </c>
+      <c r="AF4" t="inlineStr">
+        <is>
+          <t>07:05</t>
+        </is>
+      </c>
+      <c r="AG4" t="inlineStr">
+        <is>
+          <t>05:32</t>
+        </is>
+      </c>
+      <c r="AH4" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI4" t="n">
+        <v>0</v>
+      </c>
       <c r="AJ4" t="inlineStr">
         <is>
           <t>W1</t>
@@ -4748,7 +4818,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J3"/>
+  <dimension ref="A1:J4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4866,6 +4936,48 @@
       <c r="J3" t="inlineStr">
         <is>
           <t>65:00</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>Rittich</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F4" t="n">
+        <v>35</v>
+      </c>
+      <c r="G4" t="n">
+        <v>29</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.829</v>
+      </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>60:00</t>
         </is>
       </c>
     </row>
@@ -5228,7 +5340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -5328,6 +5440,26 @@
       <c r="B10" t="inlineStr">
         <is>
           <t>Three straight NYI minors in the 1st of G2 vs. NJD put New Jersey two men up twice, and the only goal of that stretch went the other way.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="n">
+        <v>2</v>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>NYI won G2 vs. NJD by five while being outshot &lt;b&gt;42-35&lt;/b&gt; and winning &lt;b&gt;14 of 46 faceoffs (30%)&lt;/b&gt;.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="n">
+        <v>2</v>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>The Isles have killed all &lt;b&gt;6&lt;/b&gt; power plays they have faced this season and are &lt;b&gt;1 for 7&lt;/b&gt; on their own, the goal coming in the 3rd of G2 vs. NJD.</t>
         </is>
       </c>
     </row>
@@ -10766,7 +10898,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:B13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -10909,6 +11041,18 @@
         </is>
       </c>
     </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>G2 vs NJD: four team-stats screens logged (1st, 2nd, final; per-period shots and hits differenced from the cumulative screens). PP 1/5 with the only goal in the 3rd confirms Cizikas' goal was even strength. Rittich went the distance: 35 SA, 29 SV. The NYI starter is still unknown - 42 SA, 41 SV, 1 GA, W is waiting on the name.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Sorokin starts by default; log his G2 win (20260908-032121)
The user's ruling: Sorokin is the starter in every game unless he names
Varlamov, and the lineup screen showing Varlamov in slot 1 does not override it.
Recorded in the manual's standing calls, so the goalie row no longer waits on a
name.

G2: 42 SA, 41 SV, 1 GA, .976, W. Season line 1-0-1, .965 on 85 shots, and the
Team Goaltending section now covers both games rather than one of two.

Recent Headlines leads with the 41 saves; the Cizikas own-goal credit comes out
to keep the section at six rows, and the recap still carries it.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gvmhg1m6TGt3JAtgHQ7SJs
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -4676,7 +4676,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K3"/>
+  <dimension ref="A1:K4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -4802,6 +4802,51 @@
         <v>0</v>
       </c>
       <c r="K3" t="inlineStr">
+        <is>
+          <t>Start</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="n">
+        <v>2</v>
+      </c>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>NJD</t>
+        </is>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>I. Sorokin</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>W</t>
+        </is>
+      </c>
+      <c r="E4" t="n">
+        <v>42</v>
+      </c>
+      <c r="F4" t="n">
+        <v>41</v>
+      </c>
+      <c r="G4" t="n">
+        <v>1</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.976</v>
+      </c>
+      <c r="I4" t="inlineStr">
+        <is>
+          <t>60:00</t>
+        </is>
+      </c>
+      <c r="J4" t="n">
+        <v>0</v>
+      </c>
+      <c r="K4" t="inlineStr">
         <is>
           <t>Start</t>
         </is>
@@ -5615,16 +5660,16 @@
         <v>2</v>
       </c>
       <c r="B7" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Points</t>
+          <t>Saves</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Schaefer&lt;/b&gt; set up the opening goal, fed Schenn on the power play and scored shorthanded himself in G2 vs. NJD, a three-point night from a 19-year-old defenseman.</t>
+          <t>&lt;b&gt;Sorokin&lt;/b&gt; was beaten only when Bratt got to his own rebound in the 2nd of G2 vs. NJD, and has allowed three goals in two starts.</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -5638,7 +5683,7 @@
         <v>2</v>
       </c>
       <c r="B8" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -5647,7 +5692,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Schenn&lt;/b&gt; found Duclair at the right post in the 1st and finished Coronato's pass from above the right circle in the 3rd of G2 vs. NJD.</t>
+          <t>&lt;b&gt;Schaefer&lt;/b&gt; set up the opening goal, fed Schenn on the power play and scored shorthanded himself in G2 vs. NJD, a three-point night from a 19-year-old defenseman.</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -5661,16 +5706,16 @@
         <v>2</v>
       </c>
       <c r="B9" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Goals</t>
+          <t>Points</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Palmieri&lt;/b&gt; one-timed Horvat's cross-slot feed from the left circle to open the scoring in G2 vs. NJD, the first of six Islanders goals.</t>
+          <t>&lt;b&gt;Schenn&lt;/b&gt; found Duclair at the right post in the 1st and finished Coronato's pass from above the right circle in the 3rd of G2 vs. NJD.</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -5684,16 +5729,16 @@
         <v>2</v>
       </c>
       <c r="B10" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Games</t>
+          <t>Goals</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Horvat&lt;/b&gt; has a point in each of the first two games: the goal in G1 at TOR and the primary assist on Palmieri's opener in G2 vs. NJD.</t>
+          <t>&lt;b&gt;Palmieri&lt;/b&gt; one-timed Horvat's cross-slot feed from the left circle to open the scoring in G2 vs. NJD, the first of six Islanders goals.</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
@@ -5707,16 +5752,16 @@
         <v>2</v>
       </c>
       <c r="B11" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Goals</t>
+          <t>Games</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Maccelli&lt;/b&gt; outran two defensemen down the slot and beat Rittich for the last of the six in G2 vs. NJD.</t>
+          <t>&lt;b&gt;Horvat&lt;/b&gt; has a point in each of the first two games: the goal in G1 at TOR and the primary assist on Palmieri's opener in G2 vs. NJD.</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
@@ -5739,7 +5784,7 @@
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>&lt;b&gt;Cizikas&lt;/b&gt; was credited in the 3rd of G2 vs. NJD after he lost the puck at the side of the net and Bratt knocked it in himself.</t>
+          <t>&lt;b&gt;Maccelli&lt;/b&gt; outran two defensemen down the slot and beat Rittich for the last of the six in G2 vs. NJD.</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
@@ -10898,7 +10943,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11053,6 +11098,18 @@
         </is>
       </c>
     </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Sorokin is the starter by default and is logged as the starting goalie in every game unless the user names Varlamov. G2: 42 SA, 41 SV, 1 GA, W.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add TOR's team ratings (20260908-032754)
Toronto 89 offense / 87 defense / 85 goaltending, off the matchup screen. Two of
32 clubs rated.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gvmhg1m6TGt3JAtgHQ7SJs
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -10821,6 +10821,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E29" t="n">
+        <v>89</v>
+      </c>
+      <c r="F29" t="n">
+        <v>87</v>
+      </c>
+      <c r="G29" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -10943,7 +10952,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B14"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11110,6 +11119,18 @@
         </is>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Team ratings: TOR 89/87/85.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Load team ratings for all 32 clubs (20260908-033557)
The remaining 30 clubs off the matchup screens, so the Team Ratings table is
complete and every column sorts on real numbers. NYI reads 87 offense / 89
defense / 93 goaltending.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gvmhg1m6TGt3JAtgHQ7SJs
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -10240,6 +10240,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E3" t="n">
+        <v>88</v>
+      </c>
+      <c r="F3" t="n">
+        <v>83</v>
+      </c>
+      <c r="G3" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -10262,6 +10271,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E4" t="n">
+        <v>88</v>
+      </c>
+      <c r="F4" t="n">
+        <v>85</v>
+      </c>
+      <c r="G4" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -10284,6 +10302,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E5" t="n">
+        <v>87</v>
+      </c>
+      <c r="F5" t="n">
+        <v>87</v>
+      </c>
+      <c r="G5" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -10306,6 +10333,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E6" t="n">
+        <v>81</v>
+      </c>
+      <c r="F6" t="n">
+        <v>85</v>
+      </c>
+      <c r="G6" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -10328,6 +10364,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E7" t="n">
+        <v>90</v>
+      </c>
+      <c r="F7" t="n">
+        <v>89</v>
+      </c>
+      <c r="G7" t="n">
+        <v>86</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -10350,6 +10395,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E8" t="n">
+        <v>85</v>
+      </c>
+      <c r="F8" t="n">
+        <v>84</v>
+      </c>
+      <c r="G8" t="n">
+        <v>86</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -10372,6 +10426,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E9" t="n">
+        <v>90</v>
+      </c>
+      <c r="F9" t="n">
+        <v>90</v>
+      </c>
+      <c r="G9" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -10394,6 +10457,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E10" t="n">
+        <v>87</v>
+      </c>
+      <c r="F10" t="n">
+        <v>87</v>
+      </c>
+      <c r="G10" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -10416,6 +10488,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E11" t="n">
+        <v>88</v>
+      </c>
+      <c r="F11" t="n">
+        <v>89</v>
+      </c>
+      <c r="G11" t="n">
+        <v>86</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -10438,6 +10519,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E12" t="n">
+        <v>85</v>
+      </c>
+      <c r="F12" t="n">
+        <v>86</v>
+      </c>
+      <c r="G12" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -10460,6 +10550,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E13" t="n">
+        <v>89</v>
+      </c>
+      <c r="F13" t="n">
+        <v>86</v>
+      </c>
+      <c r="G13" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -10482,6 +10581,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E14" t="n">
+        <v>91</v>
+      </c>
+      <c r="F14" t="n">
+        <v>87</v>
+      </c>
+      <c r="G14" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -10504,6 +10612,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E15" t="n">
+        <v>89</v>
+      </c>
+      <c r="F15" t="n">
+        <v>85</v>
+      </c>
+      <c r="G15" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -10526,6 +10643,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E16" t="n">
+        <v>86</v>
+      </c>
+      <c r="F16" t="n">
+        <v>89</v>
+      </c>
+      <c r="G16" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -10548,6 +10674,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E17" t="n">
+        <v>91</v>
+      </c>
+      <c r="F17" t="n">
+        <v>88</v>
+      </c>
+      <c r="G17" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -10570,6 +10705,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E18" t="n">
+        <v>87</v>
+      </c>
+      <c r="F18" t="n">
+        <v>84</v>
+      </c>
+      <c r="G18" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -10623,6 +10767,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E20" t="n">
+        <v>87</v>
+      </c>
+      <c r="F20" t="n">
+        <v>89</v>
+      </c>
+      <c r="G20" t="n">
+        <v>93</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -10645,6 +10798,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E21" t="n">
+        <v>85</v>
+      </c>
+      <c r="F21" t="n">
+        <v>87</v>
+      </c>
+      <c r="G21" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -10667,6 +10829,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E22" t="n">
+        <v>90</v>
+      </c>
+      <c r="F22" t="n">
+        <v>83</v>
+      </c>
+      <c r="G22" t="n">
+        <v>84</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -10689,6 +10860,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E23" t="n">
+        <v>87</v>
+      </c>
+      <c r="F23" t="n">
+        <v>84</v>
+      </c>
+      <c r="G23" t="n">
+        <v>87</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -10711,6 +10891,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E24" t="n">
+        <v>90</v>
+      </c>
+      <c r="F24" t="n">
+        <v>84</v>
+      </c>
+      <c r="G24" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -10733,6 +10922,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E25" t="n">
+        <v>87</v>
+      </c>
+      <c r="F25" t="n">
+        <v>82</v>
+      </c>
+      <c r="G25" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -10755,6 +10953,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E26" t="n">
+        <v>86</v>
+      </c>
+      <c r="F26" t="n">
+        <v>85</v>
+      </c>
+      <c r="G26" t="n">
+        <v>83</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -10777,6 +10984,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E27" t="n">
+        <v>86</v>
+      </c>
+      <c r="F27" t="n">
+        <v>84</v>
+      </c>
+      <c r="G27" t="n">
+        <v>85</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -10799,6 +11015,15 @@
           <t>Atlantic</t>
         </is>
       </c>
+      <c r="E28" t="n">
+        <v>89</v>
+      </c>
+      <c r="F28" t="n">
+        <v>88</v>
+      </c>
+      <c r="G28" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -10852,6 +11077,15 @@
           <t>Central</t>
         </is>
       </c>
+      <c r="E30" t="n">
+        <v>89</v>
+      </c>
+      <c r="F30" t="n">
+        <v>83</v>
+      </c>
+      <c r="G30" t="n">
+        <v>78</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -10874,6 +11108,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E31" t="n">
+        <v>84</v>
+      </c>
+      <c r="F31" t="n">
+        <v>81</v>
+      </c>
+      <c r="G31" t="n">
+        <v>86</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -10896,6 +11139,15 @@
           <t>Pacific</t>
         </is>
       </c>
+      <c r="E32" t="n">
+        <v>87</v>
+      </c>
+      <c r="F32" t="n">
+        <v>89</v>
+      </c>
+      <c r="G32" t="n">
+        <v>82</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -10918,6 +11170,15 @@
           <t>Metropolitan</t>
         </is>
       </c>
+      <c r="E33" t="n">
+        <v>91</v>
+      </c>
+      <c r="F33" t="n">
+        <v>86</v>
+      </c>
+      <c r="G33" t="n">
+        <v>89</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -10939,6 +11200,15 @@
         <is>
           <t>Central</t>
         </is>
+      </c>
+      <c r="E34" t="n">
+        <v>86</v>
+      </c>
+      <c r="F34" t="n">
+        <v>86</v>
+      </c>
+      <c r="G34" t="n">
+        <v>92</v>
       </c>
     </row>
   </sheetData>
@@ -10952,7 +11222,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -11131,6 +11401,18 @@
         </is>
       </c>
     </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>10/03/2026</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Team ratings loaded for the remaining 30 clubs from the user's report; all 32 are now rated. NYI reads 87 offense / 89 defense / 93 goaltending.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Revert Passed to Declined on waivers (20260912-024502)
"Passed" is not the word the game or the sport uses for a waiver a club does
not claim - Declined is - and coining it was freelancing. The Deslauriers row
goes back to Declined; the claim keeps Claimed, and an assignment keeps "-".

Recorded in S7: vocabulary comes from the game and the sport, never from what
reads better. If the screen or the sport has a word for something, that is the
word; if neither does, ask rather than coin one.

The meta reads "5 logged, 3 declined, 1 claimed" again, and every word in it is
still an actual Result value.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01KxzpKYmvBdgFq1wUx73qDq
</commit_message>
<xml_diff>
--- a/S1 NY Islanders.xlsx
+++ b/S1 NY Islanders.xlsx
@@ -7006,7 +7006,7 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Passed</t>
+          <t>Declined</t>
         </is>
       </c>
     </row>
@@ -12333,7 +12333,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -12664,7 +12664,19 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Transactions Result vocabulary is per Type: a Trade offer is Accepted / Declined, a Waivers row is Claimed / Passed, and an Assignment is '-' because a roster move has no accept-or-decline outcome to report - the same reason its Partner column holds '-' on a waiver claim.</t>
+          <t>Transactions Result vocabulary is per Type: a Trade offer is Accepted / Declined, a Waivers row is Claimed / Declined, and an Assignment is '-' because a roster move has no accept-or-decline outcome to report - the same reason its Partner column holds '-' on a waiver claim.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>10/06/2026</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>'Passed' was not the game's word for a waiver a club does not claim - Declined is. The Result column takes the vocabulary the game and the sport use, never a synonym that reads better.</t>
         </is>
       </c>
     </row>

</xml_diff>